<commit_message>
Revert "Merge branch 'main' of https://github.com/tt800w/contratos1"
This reverts commit 56418792ae76bbd06e1526c78cd6f01088223790, reversing
changes made to aa68b20286f49cb080bb57be3adea534e859c599.
</commit_message>
<xml_diff>
--- a/dist/contratos/Excel prueba de contrato.xlsx
+++ b/dist/contratos/Excel prueba de contrato.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Campuslands\contratos1\public\contratos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\QM\Desktop\contratos1\public\contratos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98BD3EFE-7ABF-4F78-AC71-7DF1FC16034B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B0A3D43-524F-45C1-9111-DC9F288C5F85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1440" yWindow="192" windowWidth="21600" windowHeight="11232" xr2:uid="{154874EA-5800-4E6F-B81B-B598FC728375}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{154874EA-5800-4E6F-B81B-B598FC728375}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -2208,7 +2208,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3267,21 +3267,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{658075FD-451C-4A05-8045-1F7769A17105}">
   <dimension ref="A1:V253"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="16.296875" customWidth="1"/>
+    <col min="2" max="2" width="16.26953125" customWidth="1"/>
     <col min="3" max="3" width="27" customWidth="1"/>
-    <col min="4" max="4" width="20.19921875" customWidth="1"/>
-    <col min="5" max="5" width="8.19921875" customWidth="1"/>
-    <col min="7" max="7" width="14.3984375" customWidth="1"/>
-    <col min="8" max="8" width="12.19921875" customWidth="1"/>
-    <col min="9" max="9" width="17.19921875" customWidth="1"/>
-    <col min="10" max="10" width="16.09765625" customWidth="1"/>
-    <col min="11" max="11" width="14.19921875" customWidth="1"/>
-    <col min="12" max="12" width="33.19921875" customWidth="1"/>
+    <col min="4" max="4" width="20.1796875" customWidth="1"/>
+    <col min="5" max="5" width="8.1796875" customWidth="1"/>
+    <col min="7" max="7" width="14.36328125" customWidth="1"/>
+    <col min="8" max="8" width="12.1796875" customWidth="1"/>
+    <col min="9" max="9" width="17.1796875" customWidth="1"/>
+    <col min="10" max="10" width="16.08984375" customWidth="1"/>
+    <col min="11" max="11" width="14.1796875" customWidth="1"/>
+    <col min="12" max="12" width="33.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="1" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3339,7 +3339,7 @@
       <c r="U1" s="4"/>
       <c r="V1" s="4"/>
     </row>
-    <row r="2" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="2" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="5"/>
       <c r="B2" s="6">
         <v>45875.555717592593</v>
@@ -3395,7 +3395,7 @@
       <c r="U2" s="11"/>
       <c r="V2" s="11"/>
     </row>
-    <row r="3" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="3" spans="1:22" ht="65.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="12"/>
       <c r="B3" s="6">
         <v>45875.599814814814</v>
@@ -3441,7 +3441,7 @@
       <c r="U3" s="11"/>
       <c r="V3" s="11"/>
     </row>
-    <row r="4" spans="1:22" ht="27" thickBot="1">
+    <row r="4" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="5"/>
       <c r="B4" s="6">
         <v>45875.603206018517</v>
@@ -3495,7 +3495,7 @@
       <c r="U4" s="11"/>
       <c r="V4" s="11"/>
     </row>
-    <row r="5" spans="1:22" ht="27" thickBot="1">
+    <row r="5" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="12"/>
       <c r="B5" s="6">
         <v>45875.626400462963</v>
@@ -3541,7 +3541,7 @@
       <c r="U5" s="11"/>
       <c r="V5" s="11"/>
     </row>
-    <row r="6" spans="1:22" ht="27" thickBot="1">
+    <row r="6" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="5"/>
       <c r="B6" s="6">
         <v>45875.63480324074</v>
@@ -3587,7 +3587,7 @@
       <c r="U6" s="11"/>
       <c r="V6" s="11"/>
     </row>
-    <row r="7" spans="1:22" ht="27" thickBot="1">
+    <row r="7" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="12"/>
       <c r="B7" s="6">
         <v>45875.636967592596</v>
@@ -3633,7 +3633,7 @@
       <c r="U7" s="11"/>
       <c r="V7" s="11"/>
     </row>
-    <row r="8" spans="1:22" ht="53.4" thickBot="1">
+    <row r="8" spans="1:22" ht="78.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="5"/>
       <c r="B8" s="6">
         <v>45875.834710648145</v>
@@ -3679,7 +3679,7 @@
       <c r="U8" s="11"/>
       <c r="V8" s="11"/>
     </row>
-    <row r="9" spans="1:22" ht="27" thickBot="1">
+    <row r="9" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="12"/>
       <c r="B9" s="6">
         <v>45877.459016203706</v>
@@ -3725,7 +3725,7 @@
       <c r="U9" s="11"/>
       <c r="V9" s="11"/>
     </row>
-    <row r="10" spans="1:22" ht="27" thickBot="1">
+    <row r="10" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="5"/>
       <c r="B10" s="6">
         <v>45877.469965277778</v>
@@ -3771,7 +3771,7 @@
       <c r="U10" s="11"/>
       <c r="V10" s="11"/>
     </row>
-    <row r="11" spans="1:22" ht="27" thickBot="1">
+    <row r="11" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="12"/>
       <c r="B11" s="6">
         <v>45877.472488425927</v>
@@ -3817,7 +3817,7 @@
       <c r="U11" s="11"/>
       <c r="V11" s="11"/>
     </row>
-    <row r="12" spans="1:22" ht="27" thickBot="1">
+    <row r="12" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="5"/>
       <c r="B12" s="6">
         <v>45877.488206018519</v>
@@ -3871,7 +3871,7 @@
       <c r="U12" s="11"/>
       <c r="V12" s="11"/>
     </row>
-    <row r="13" spans="1:22" ht="66.599999999999994" thickBot="1">
+    <row r="13" spans="1:22" ht="91.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="12"/>
       <c r="B13" s="6">
         <v>45878.374050925922</v>
@@ -3917,7 +3917,7 @@
       <c r="U13" s="11"/>
       <c r="V13" s="11"/>
     </row>
-    <row r="14" spans="1:22" ht="27" thickBot="1">
+    <row r="14" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="5"/>
       <c r="B14" s="6">
         <v>45878.374664351853</v>
@@ -3971,7 +3971,7 @@
       <c r="U14" s="11"/>
       <c r="V14" s="11"/>
     </row>
-    <row r="15" spans="1:22" ht="27" thickBot="1">
+    <row r="15" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="12"/>
       <c r="B15" s="6">
         <v>45878.375868055555</v>
@@ -4017,7 +4017,7 @@
       <c r="U15" s="11"/>
       <c r="V15" s="11"/>
     </row>
-    <row r="16" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="16" spans="1:22" ht="65.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="5"/>
       <c r="B16" s="6">
         <v>45878.384502314817</v>
@@ -4071,7 +4071,7 @@
       <c r="U16" s="11"/>
       <c r="V16" s="11"/>
     </row>
-    <row r="17" spans="1:22" ht="27" thickBot="1">
+    <row r="17" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="23"/>
       <c r="B17" s="24">
         <v>45878.391921296294</v>
@@ -4117,7 +4117,7 @@
       <c r="U17" s="11"/>
       <c r="V17" s="11"/>
     </row>
-    <row r="18" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="18" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="5"/>
       <c r="B18" s="6">
         <v>45878.406574074077</v>
@@ -4163,7 +4163,7 @@
       <c r="U18" s="11"/>
       <c r="V18" s="11"/>
     </row>
-    <row r="19" spans="1:22" ht="27" thickBot="1">
+    <row r="19" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="12"/>
       <c r="B19" s="6">
         <v>45878.428078703706</v>
@@ -4209,7 +4209,7 @@
       <c r="U19" s="11"/>
       <c r="V19" s="11"/>
     </row>
-    <row r="20" spans="1:22" ht="27" thickBot="1">
+    <row r="20" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="5"/>
       <c r="B20" s="6">
         <v>45878.464918981481</v>
@@ -4255,7 +4255,7 @@
       <c r="U20" s="11"/>
       <c r="V20" s="11"/>
     </row>
-    <row r="21" spans="1:22" ht="27" thickBot="1">
+    <row r="21" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="23"/>
       <c r="B21" s="24">
         <v>45878.474409722221</v>
@@ -4301,7 +4301,7 @@
       <c r="U21" s="11"/>
       <c r="V21" s="11"/>
     </row>
-    <row r="22" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="22" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="5"/>
       <c r="B22" s="6">
         <v>45878.474652777775</v>
@@ -4355,7 +4355,7 @@
       <c r="U22" s="11"/>
       <c r="V22" s="11"/>
     </row>
-    <row r="23" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="23" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="12"/>
       <c r="B23" s="6">
         <v>45878.489317129628</v>
@@ -4401,7 +4401,7 @@
       <c r="U23" s="11"/>
       <c r="V23" s="11"/>
     </row>
-    <row r="24" spans="1:22" ht="27" thickBot="1">
+    <row r="24" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="5"/>
       <c r="B24" s="6">
         <v>45878.503067129626</v>
@@ -4447,7 +4447,7 @@
       <c r="U24" s="11"/>
       <c r="V24" s="11"/>
     </row>
-    <row r="25" spans="1:22" ht="27" thickBot="1">
+    <row r="25" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="12"/>
       <c r="B25" s="6">
         <v>45879.828877314816</v>
@@ -4493,7 +4493,7 @@
       <c r="U25" s="11"/>
       <c r="V25" s="11"/>
     </row>
-    <row r="26" spans="1:22" ht="27" thickBot="1">
+    <row r="26" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="5"/>
       <c r="B26" s="6">
         <v>45879.896458333336</v>
@@ -4539,7 +4539,7 @@
       <c r="U26" s="11"/>
       <c r="V26" s="11"/>
     </row>
-    <row r="27" spans="1:22" ht="27" thickBot="1">
+    <row r="27" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="12"/>
       <c r="B27" s="6">
         <v>45880.520821759259</v>
@@ -4585,7 +4585,7 @@
       <c r="U27" s="11"/>
       <c r="V27" s="11"/>
     </row>
-    <row r="28" spans="1:22" ht="27" thickBot="1">
+    <row r="28" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="5"/>
       <c r="B28" s="6">
         <v>45880.523761574077</v>
@@ -4631,7 +4631,7 @@
       <c r="U28" s="11"/>
       <c r="V28" s="11"/>
     </row>
-    <row r="29" spans="1:22" ht="27" thickBot="1">
+    <row r="29" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="12"/>
       <c r="B29" s="6">
         <v>45880.525300925925</v>
@@ -4677,7 +4677,7 @@
       <c r="U29" s="11"/>
       <c r="V29" s="11"/>
     </row>
-    <row r="30" spans="1:22" ht="27" thickBot="1">
+    <row r="30" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="5"/>
       <c r="B30" s="6">
         <v>45880.528229166666</v>
@@ -4723,7 +4723,7 @@
       <c r="U30" s="11"/>
       <c r="V30" s="11"/>
     </row>
-    <row r="31" spans="1:22" ht="27" thickBot="1">
+    <row r="31" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="12"/>
       <c r="B31" s="6">
         <v>45880.536585648151</v>
@@ -4769,7 +4769,7 @@
       <c r="U31" s="11"/>
       <c r="V31" s="11"/>
     </row>
-    <row r="32" spans="1:22" ht="27" thickBot="1">
+    <row r="32" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="5"/>
       <c r="B32" s="6">
         <v>45880.539039351854</v>
@@ -4815,7 +4815,7 @@
       <c r="U32" s="11"/>
       <c r="V32" s="11"/>
     </row>
-    <row r="33" spans="1:22" ht="27" thickBot="1">
+    <row r="33" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="12"/>
       <c r="B33" s="6">
         <v>45880.549201388887</v>
@@ -4861,7 +4861,7 @@
       <c r="U33" s="11"/>
       <c r="V33" s="11"/>
     </row>
-    <row r="34" spans="1:22" ht="27" thickBot="1">
+    <row r="34" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="5"/>
       <c r="B34" s="6">
         <v>45880.551805555559</v>
@@ -4907,7 +4907,7 @@
       <c r="U34" s="11"/>
       <c r="V34" s="11"/>
     </row>
-    <row r="35" spans="1:22" ht="27" thickBot="1">
+    <row r="35" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="12"/>
       <c r="B35" s="6">
         <v>45880.552766203706</v>
@@ -4953,7 +4953,7 @@
       <c r="U35" s="11"/>
       <c r="V35" s="11"/>
     </row>
-    <row r="36" spans="1:22" ht="53.4" thickBot="1">
+    <row r="36" spans="1:22" ht="65.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A36" s="5"/>
       <c r="B36" s="6">
         <v>45880.569918981484</v>
@@ -4999,7 +4999,7 @@
       <c r="U36" s="11"/>
       <c r="V36" s="11"/>
     </row>
-    <row r="37" spans="1:22" ht="27" thickBot="1">
+    <row r="37" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="12"/>
       <c r="B37" s="6">
         <v>45880.603148148148</v>
@@ -5045,7 +5045,7 @@
       <c r="U37" s="11"/>
       <c r="V37" s="11"/>
     </row>
-    <row r="38" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="38" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="5"/>
       <c r="B38" s="6">
         <v>45880.797442129631</v>
@@ -5099,7 +5099,7 @@
       <c r="U38" s="11"/>
       <c r="V38" s="11"/>
     </row>
-    <row r="39" spans="1:22" ht="27" thickBot="1">
+    <row r="39" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="12"/>
       <c r="B39" s="6">
         <v>45881.493460648147</v>
@@ -5145,7 +5145,7 @@
       <c r="U39" s="11"/>
       <c r="V39" s="11"/>
     </row>
-    <row r="40" spans="1:22" ht="27" thickBot="1">
+    <row r="40" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="5"/>
       <c r="B40" s="6">
         <v>45881.509502314817</v>
@@ -5199,7 +5199,7 @@
       <c r="U40" s="11"/>
       <c r="V40" s="11"/>
     </row>
-    <row r="41" spans="1:22" ht="27" thickBot="1">
+    <row r="41" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="12"/>
       <c r="B41" s="6">
         <v>45881.621203703704</v>
@@ -5253,7 +5253,7 @@
       <c r="U41" s="11"/>
       <c r="V41" s="11"/>
     </row>
-    <row r="42" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="42" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="5"/>
       <c r="B42" s="6">
         <v>45881.937615740739</v>
@@ -5299,7 +5299,7 @@
       <c r="U42" s="11"/>
       <c r="V42" s="11"/>
     </row>
-    <row r="43" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="43" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A43" s="12"/>
       <c r="B43" s="6">
         <v>45881.966354166667</v>
@@ -5353,7 +5353,7 @@
       <c r="U43" s="11"/>
       <c r="V43" s="11"/>
     </row>
-    <row r="44" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="44" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A44" s="5"/>
       <c r="B44" s="6">
         <v>45882.207835648151</v>
@@ -5407,7 +5407,7 @@
       <c r="U44" s="11"/>
       <c r="V44" s="11"/>
     </row>
-    <row r="45" spans="1:22" ht="27" thickBot="1">
+    <row r="45" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A45" s="12"/>
       <c r="B45" s="6">
         <v>45882.706354166665</v>
@@ -5453,7 +5453,7 @@
       <c r="U45" s="11"/>
       <c r="V45" s="11"/>
     </row>
-    <row r="46" spans="1:22" ht="27" thickBot="1">
+    <row r="46" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="5"/>
       <c r="B46" s="6">
         <v>45883.70884259259</v>
@@ -5499,7 +5499,7 @@
       <c r="U46" s="11"/>
       <c r="V46" s="11"/>
     </row>
-    <row r="47" spans="1:22" ht="27" thickBot="1">
+    <row r="47" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A47" s="12"/>
       <c r="B47" s="6">
         <v>45883.780763888892</v>
@@ -5545,7 +5545,7 @@
       <c r="U47" s="11"/>
       <c r="V47" s="11"/>
     </row>
-    <row r="48" spans="1:22" ht="27" thickBot="1">
+    <row r="48" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A48" s="5"/>
       <c r="B48" s="6">
         <v>45884.710613425923</v>
@@ -5591,7 +5591,7 @@
       <c r="U48" s="11"/>
       <c r="V48" s="11"/>
     </row>
-    <row r="49" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="49" spans="1:22" ht="65.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="12"/>
       <c r="B49" s="6">
         <v>45888.419664351852</v>
@@ -5645,7 +5645,7 @@
       <c r="U49" s="11"/>
       <c r="V49" s="11"/>
     </row>
-    <row r="50" spans="1:22" ht="27" thickBot="1">
+    <row r="50" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A50" s="5"/>
       <c r="B50" s="6">
         <v>45888.428136574075</v>
@@ -5691,7 +5691,7 @@
       <c r="U50" s="11"/>
       <c r="V50" s="11"/>
     </row>
-    <row r="51" spans="1:22" ht="27" thickBot="1">
+    <row r="51" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A51" s="12"/>
       <c r="B51" s="6">
         <v>45888.428761574076</v>
@@ -5737,7 +5737,7 @@
       <c r="U51" s="11"/>
       <c r="V51" s="11"/>
     </row>
-    <row r="52" spans="1:22" ht="27" thickBot="1">
+    <row r="52" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A52" s="30"/>
       <c r="B52" s="31">
         <v>45888.470763888887</v>
@@ -5783,7 +5783,7 @@
       <c r="U52" s="11"/>
       <c r="V52" s="11"/>
     </row>
-    <row r="53" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="53" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A53" s="12"/>
       <c r="B53" s="6">
         <v>45888.482407407406</v>
@@ -5829,7 +5829,7 @@
       <c r="U53" s="11"/>
       <c r="V53" s="11"/>
     </row>
-    <row r="54" spans="1:22" ht="27" thickBot="1">
+    <row r="54" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A54" s="5"/>
       <c r="B54" s="6">
         <v>45888.550613425927</v>
@@ -5875,7 +5875,7 @@
       <c r="U54" s="11"/>
       <c r="V54" s="11"/>
     </row>
-    <row r="55" spans="1:22" ht="27" thickBot="1">
+    <row r="55" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A55" s="34"/>
       <c r="B55" s="35">
         <v>45889.478055555555</v>
@@ -5921,7 +5921,7 @@
       <c r="U55" s="11"/>
       <c r="V55" s="11"/>
     </row>
-    <row r="56" spans="1:22" ht="27" thickBot="1">
+    <row r="56" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="5"/>
       <c r="B56" s="6">
         <v>45889.744629629633</v>
@@ -5967,7 +5967,7 @@
       <c r="U56" s="11"/>
       <c r="V56" s="11"/>
     </row>
-    <row r="57" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="57" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A57" s="12"/>
       <c r="B57" s="6">
         <v>45891.716238425928</v>
@@ -6013,7 +6013,7 @@
       <c r="U57" s="11"/>
       <c r="V57" s="11"/>
     </row>
-    <row r="58" spans="1:22" ht="27" thickBot="1">
+    <row r="58" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A58" s="5"/>
       <c r="B58" s="6">
         <v>45895.757743055554</v>
@@ -6059,7 +6059,7 @@
       <c r="U58" s="11"/>
       <c r="V58" s="11"/>
     </row>
-    <row r="59" spans="1:22" ht="14.4" thickBot="1">
+    <row r="59" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A59" s="12"/>
       <c r="B59" s="6">
         <v>45895.761284722219</v>
@@ -6105,7 +6105,7 @@
       <c r="U59" s="11"/>
       <c r="V59" s="11"/>
     </row>
-    <row r="60" spans="1:22" ht="27" thickBot="1">
+    <row r="60" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A60" s="30"/>
       <c r="B60" s="36">
         <v>45896.566030092596</v>
@@ -6151,7 +6151,7 @@
       <c r="U60" s="11"/>
       <c r="V60" s="11"/>
     </row>
-    <row r="61" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="61" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="34"/>
       <c r="B61" s="38">
         <v>45896.653113425928</v>
@@ -6205,7 +6205,7 @@
       <c r="U61" s="11"/>
       <c r="V61" s="11"/>
     </row>
-    <row r="62" spans="1:22" ht="27" thickBot="1">
+    <row r="62" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A62" s="40"/>
       <c r="B62" s="41">
         <v>45898.71434027778</v>
@@ -6251,7 +6251,7 @@
       <c r="U62" s="11"/>
       <c r="V62" s="11"/>
     </row>
-    <row r="63" spans="1:22" ht="27" thickBot="1">
+    <row r="63" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A63" s="12"/>
       <c r="B63" s="6">
         <v>45904.006249999999</v>
@@ -6297,7 +6297,7 @@
       <c r="U63" s="11"/>
       <c r="V63" s="11"/>
     </row>
-    <row r="64" spans="1:22" ht="27" thickBot="1">
+    <row r="64" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A64" s="42" t="s">
         <v>301</v>
       </c>
@@ -6345,7 +6345,7 @@
       <c r="U64" s="11"/>
       <c r="V64" s="11"/>
     </row>
-    <row r="65" spans="1:22" ht="27" thickBot="1">
+    <row r="65" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A65" s="43" t="s">
         <v>301</v>
       </c>
@@ -6393,7 +6393,7 @@
       <c r="U65" s="11"/>
       <c r="V65" s="11"/>
     </row>
-    <row r="66" spans="1:22" ht="27" thickBot="1">
+    <row r="66" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A66" s="42" t="s">
         <v>301</v>
       </c>
@@ -6441,7 +6441,7 @@
       <c r="U66" s="11"/>
       <c r="V66" s="11"/>
     </row>
-    <row r="67" spans="1:22" ht="27" thickBot="1">
+    <row r="67" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A67" s="43" t="s">
         <v>301</v>
       </c>
@@ -6489,7 +6489,7 @@
       <c r="U67" s="11"/>
       <c r="V67" s="11"/>
     </row>
-    <row r="68" spans="1:22" ht="27" thickBot="1">
+    <row r="68" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A68" s="42" t="s">
         <v>301</v>
       </c>
@@ -6537,7 +6537,7 @@
       <c r="U68" s="11"/>
       <c r="V68" s="11"/>
     </row>
-    <row r="69" spans="1:22" ht="27" thickBot="1">
+    <row r="69" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A69" s="43" t="s">
         <v>301</v>
       </c>
@@ -6585,7 +6585,7 @@
       <c r="U69" s="11"/>
       <c r="V69" s="11"/>
     </row>
-    <row r="70" spans="1:22" ht="27" thickBot="1">
+    <row r="70" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A70" s="42" t="s">
         <v>301</v>
       </c>
@@ -6633,7 +6633,7 @@
       <c r="U70" s="11"/>
       <c r="V70" s="11"/>
     </row>
-    <row r="71" spans="1:22" ht="27" thickBot="1">
+    <row r="71" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A71" s="43" t="s">
         <v>301</v>
       </c>
@@ -6681,7 +6681,7 @@
       <c r="U71" s="11"/>
       <c r="V71" s="11"/>
     </row>
-    <row r="72" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="72" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A72" s="42" t="s">
         <v>335</v>
       </c>
@@ -6737,7 +6737,7 @@
       <c r="U72" s="11"/>
       <c r="V72" s="11"/>
     </row>
-    <row r="73" spans="1:22" ht="27" thickBot="1">
+    <row r="73" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A73" s="43" t="s">
         <v>335</v>
       </c>
@@ -6785,7 +6785,7 @@
       <c r="U73" s="11"/>
       <c r="V73" s="11"/>
     </row>
-    <row r="74" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="74" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A74" s="42" t="s">
         <v>335</v>
       </c>
@@ -6841,7 +6841,7 @@
       <c r="U74" s="11"/>
       <c r="V74" s="11"/>
     </row>
-    <row r="75" spans="1:22" ht="27" thickBot="1">
+    <row r="75" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A75" s="43" t="s">
         <v>335</v>
       </c>
@@ -6889,7 +6889,7 @@
       <c r="U75" s="11"/>
       <c r="V75" s="11"/>
     </row>
-    <row r="76" spans="1:22" ht="27" thickBot="1">
+    <row r="76" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A76" s="42" t="s">
         <v>335</v>
       </c>
@@ -6945,7 +6945,7 @@
       <c r="U76" s="11"/>
       <c r="V76" s="11"/>
     </row>
-    <row r="77" spans="1:22" ht="53.4" thickBot="1">
+    <row r="77" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A77" s="43" t="s">
         <v>335</v>
       </c>
@@ -6993,7 +6993,7 @@
       <c r="U77" s="11"/>
       <c r="V77" s="11"/>
     </row>
-    <row r="78" spans="1:22" ht="27" thickBot="1">
+    <row r="78" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" s="42" t="s">
         <v>335</v>
       </c>
@@ -7041,7 +7041,7 @@
       <c r="U78" s="11"/>
       <c r="V78" s="11"/>
     </row>
-    <row r="79" spans="1:22" ht="27" thickBot="1">
+    <row r="79" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A79" s="43" t="s">
         <v>335</v>
       </c>
@@ -7097,7 +7097,7 @@
       <c r="U79" s="11"/>
       <c r="V79" s="11"/>
     </row>
-    <row r="80" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="80" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A80" s="42" t="s">
         <v>335</v>
       </c>
@@ -7145,7 +7145,7 @@
       <c r="U80" s="11"/>
       <c r="V80" s="11"/>
     </row>
-    <row r="81" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="81" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A81" s="44" t="s">
         <v>335</v>
       </c>
@@ -7201,7 +7201,7 @@
       <c r="U81" s="11"/>
       <c r="V81" s="11"/>
     </row>
-    <row r="82" spans="1:22" ht="27" thickBot="1">
+    <row r="82" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A82" s="42" t="s">
         <v>335</v>
       </c>
@@ -7249,7 +7249,7 @@
       <c r="U82" s="11"/>
       <c r="V82" s="11"/>
     </row>
-    <row r="83" spans="1:22" ht="27" thickBot="1">
+    <row r="83" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A83" s="12"/>
       <c r="B83" s="6">
         <v>45993.637881944444</v>
@@ -7295,7 +7295,7 @@
       <c r="U83" s="11"/>
       <c r="V83" s="11"/>
     </row>
-    <row r="84" spans="1:22" ht="27" thickBot="1">
+    <row r="84" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A84" s="5"/>
       <c r="B84" s="6">
         <v>45993.638310185182</v>
@@ -7341,7 +7341,7 @@
       <c r="U84" s="11"/>
       <c r="V84" s="11"/>
     </row>
-    <row r="85" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="85" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A85" s="12"/>
       <c r="B85" s="6">
         <v>45993.675069444442</v>
@@ -7395,7 +7395,7 @@
       <c r="U85" s="11"/>
       <c r="V85" s="11"/>
     </row>
-    <row r="86" spans="1:22" ht="27" thickBot="1">
+    <row r="86" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A86" s="5"/>
       <c r="B86" s="6">
         <v>45993.681030092594</v>
@@ -7441,7 +7441,7 @@
       <c r="U86" s="11"/>
       <c r="V86" s="11"/>
     </row>
-    <row r="87" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="87" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A87" s="23"/>
       <c r="B87" s="24">
         <v>45994.368032407408</v>
@@ -7495,7 +7495,7 @@
       <c r="U87" s="11"/>
       <c r="V87" s="11"/>
     </row>
-    <row r="88" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="88" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A88" s="5"/>
       <c r="B88" s="6">
         <v>46002.732037037036</v>
@@ -7541,7 +7541,7 @@
       <c r="U88" s="11"/>
       <c r="V88" s="11"/>
     </row>
-    <row r="89" spans="1:22" ht="14.4" thickBot="1">
+    <row r="89" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A89" s="12"/>
       <c r="B89" s="6">
         <v>46006.580497685187</v>
@@ -7587,7 +7587,7 @@
       <c r="U89" s="11"/>
       <c r="V89" s="11"/>
     </row>
-    <row r="90" spans="1:22" ht="27" thickBot="1">
+    <row r="90" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A90" s="5"/>
       <c r="B90" s="6">
         <v>46006.730567129627</v>
@@ -7641,7 +7641,7 @@
       <c r="U90" s="11"/>
       <c r="V90" s="11"/>
     </row>
-    <row r="91" spans="1:22" ht="27" thickBot="1">
+    <row r="91" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A91" s="12"/>
       <c r="B91" s="6">
         <v>46006.730833333335</v>
@@ -7687,7 +7687,7 @@
       <c r="U91" s="11"/>
       <c r="V91" s="11"/>
     </row>
-    <row r="92" spans="1:22" ht="27" thickBot="1">
+    <row r="92" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A92" s="5"/>
       <c r="B92" s="6">
         <v>46006.732789351852</v>
@@ -7741,7 +7741,7 @@
       <c r="U92" s="11"/>
       <c r="V92" s="11"/>
     </row>
-    <row r="93" spans="1:22" ht="27" thickBot="1">
+    <row r="93" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A93" s="12"/>
       <c r="B93" s="45">
         <v>46006.732881944445</v>
@@ -7787,7 +7787,7 @@
       <c r="U93" s="11"/>
       <c r="V93" s="11"/>
     </row>
-    <row r="94" spans="1:22" ht="27" thickBot="1">
+    <row r="94" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A94" s="46"/>
       <c r="B94" s="47">
         <v>46006.733865740738</v>
@@ -7841,7 +7841,7 @@
       <c r="U94" s="11"/>
       <c r="V94" s="11"/>
     </row>
-    <row r="95" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="95" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A95" s="12"/>
       <c r="B95" s="45">
         <v>46006.750949074078</v>
@@ -7895,7 +7895,7 @@
       <c r="U95" s="11"/>
       <c r="V95" s="11"/>
     </row>
-    <row r="96" spans="1:22" ht="27" thickBot="1">
+    <row r="96" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A96" s="46"/>
       <c r="B96" s="47">
         <v>46006.753113425926</v>
@@ -7941,7 +7941,7 @@
       <c r="U96" s="11"/>
       <c r="V96" s="11"/>
     </row>
-    <row r="97" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="97" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A97" s="12"/>
       <c r="B97" s="6">
         <v>46006.757071759261</v>
@@ -7995,7 +7995,7 @@
       <c r="U97" s="11"/>
       <c r="V97" s="11"/>
     </row>
-    <row r="98" spans="1:22" ht="53.4" thickBot="1">
+    <row r="98" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A98" s="5"/>
       <c r="B98" s="6">
         <v>46006.762337962966</v>
@@ -8049,7 +8049,7 @@
       <c r="U98" s="11"/>
       <c r="V98" s="11"/>
     </row>
-    <row r="99" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="99" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A99" s="12"/>
       <c r="B99" s="6">
         <v>46006.769791666666</v>
@@ -8103,7 +8103,7 @@
       <c r="U99" s="11"/>
       <c r="V99" s="11"/>
     </row>
-    <row r="100" spans="1:22" ht="27" thickBot="1">
+    <row r="100" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A100" s="5"/>
       <c r="B100" s="6">
         <v>46006.77516203704</v>
@@ -8149,7 +8149,7 @@
       <c r="U100" s="11"/>
       <c r="V100" s="11"/>
     </row>
-    <row r="101" spans="1:22" ht="27" thickBot="1">
+    <row r="101" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A101" s="12"/>
       <c r="B101" s="6">
         <v>46006.781215277777</v>
@@ -8203,7 +8203,7 @@
       <c r="U101" s="11"/>
       <c r="V101" s="11"/>
     </row>
-    <row r="102" spans="1:22" ht="27" thickBot="1">
+    <row r="102" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A102" s="5"/>
       <c r="B102" s="6">
         <v>46006.829513888886</v>
@@ -8249,7 +8249,7 @@
       <c r="U102" s="11"/>
       <c r="V102" s="11"/>
     </row>
-    <row r="103" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="103" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A103" s="12"/>
       <c r="B103" s="6">
         <v>46006.832638888889</v>
@@ -8295,7 +8295,7 @@
       <c r="U103" s="11"/>
       <c r="V103" s="11"/>
     </row>
-    <row r="104" spans="1:22" ht="27" thickBot="1">
+    <row r="104" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A104" s="5"/>
       <c r="B104" s="6">
         <v>46006.890879629631</v>
@@ -8341,7 +8341,7 @@
       <c r="U104" s="11"/>
       <c r="V104" s="11"/>
     </row>
-    <row r="105" spans="1:22" ht="27" thickBot="1">
+    <row r="105" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A105" s="12"/>
       <c r="B105" s="6">
         <v>46006.891736111109</v>
@@ -8387,7 +8387,7 @@
       <c r="U105" s="11"/>
       <c r="V105" s="11"/>
     </row>
-    <row r="106" spans="1:22" ht="27" thickBot="1">
+    <row r="106" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A106" s="5"/>
       <c r="B106" s="6">
         <v>46006.919062499997</v>
@@ -8433,7 +8433,7 @@
       <c r="U106" s="11"/>
       <c r="V106" s="11"/>
     </row>
-    <row r="107" spans="1:22" ht="27" thickBot="1">
+    <row r="107" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A107" s="12"/>
       <c r="B107" s="48">
         <v>46006.92559027778</v>
@@ -8487,7 +8487,7 @@
       <c r="U107" s="11"/>
       <c r="V107" s="11"/>
     </row>
-    <row r="108" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="108" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A108" s="5"/>
       <c r="B108" s="6">
         <v>46006.944386574076</v>
@@ -8541,7 +8541,7 @@
       <c r="U108" s="11"/>
       <c r="V108" s="11"/>
     </row>
-    <row r="109" spans="1:22" ht="53.4" thickBot="1">
+    <row r="109" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A109" s="12"/>
       <c r="B109" s="6">
         <v>46006.96166666667</v>
@@ -8595,7 +8595,7 @@
       <c r="U109" s="11"/>
       <c r="V109" s="11"/>
     </row>
-    <row r="110" spans="1:22" ht="27" thickBot="1">
+    <row r="110" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A110" s="5"/>
       <c r="B110" s="6">
         <v>46006.97378472222</v>
@@ -8641,7 +8641,7 @@
       <c r="U110" s="11"/>
       <c r="V110" s="11"/>
     </row>
-    <row r="111" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="111" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A111" s="12"/>
       <c r="B111" s="6">
         <v>46007.1796412037</v>
@@ -8695,7 +8695,7 @@
       <c r="U111" s="11"/>
       <c r="V111" s="11"/>
     </row>
-    <row r="112" spans="1:22" ht="27" thickBot="1">
+    <row r="112" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A112" s="5"/>
       <c r="B112" s="6">
         <v>46007.206076388888</v>
@@ -8749,7 +8749,7 @@
       <c r="U112" s="11"/>
       <c r="V112" s="11"/>
     </row>
-    <row r="113" spans="1:22" ht="53.4" thickBot="1">
+    <row r="113" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A113" s="12"/>
       <c r="B113" s="6">
         <v>46007.251354166663</v>
@@ -8803,7 +8803,7 @@
       <c r="U113" s="11"/>
       <c r="V113" s="11"/>
     </row>
-    <row r="114" spans="1:22" ht="27" thickBot="1">
+    <row r="114" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A114" s="5"/>
       <c r="B114" s="6">
         <v>46007.323703703703</v>
@@ -8857,7 +8857,7 @@
       <c r="U114" s="11"/>
       <c r="V114" s="11"/>
     </row>
-    <row r="115" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="115" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A115" s="12"/>
       <c r="B115" s="6">
         <v>46007.403368055559</v>
@@ -8911,7 +8911,7 @@
       <c r="U115" s="11"/>
       <c r="V115" s="11"/>
     </row>
-    <row r="116" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="116" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A116" s="5"/>
       <c r="B116" s="6">
         <v>46014.57371527778</v>
@@ -8965,7 +8965,7 @@
       <c r="U116" s="11"/>
       <c r="V116" s="11"/>
     </row>
-    <row r="117" spans="1:22" ht="27" thickBot="1">
+    <row r="117" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A117" s="12"/>
       <c r="B117" s="6">
         <v>46014.586192129631</v>
@@ -9019,7 +9019,7 @@
       <c r="U117" s="11"/>
       <c r="V117" s="11"/>
     </row>
-    <row r="118" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="118" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A118" s="5"/>
       <c r="B118" s="6">
         <v>46049.920532407406</v>
@@ -9073,7 +9073,7 @@
       <c r="U118" s="11"/>
       <c r="V118" s="11"/>
     </row>
-    <row r="119" spans="1:22" ht="27" thickBot="1">
+    <row r="119" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A119" s="12"/>
       <c r="B119" s="6">
         <v>46050.426030092596</v>
@@ -9127,7 +9127,7 @@
       <c r="U119" s="11"/>
       <c r="V119" s="11"/>
     </row>
-    <row r="120" spans="1:22" ht="27" thickBot="1">
+    <row r="120" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A120" s="5"/>
       <c r="B120" s="6">
         <v>46050.494062500002</v>
@@ -9173,7 +9173,7 @@
       <c r="U120" s="11"/>
       <c r="V120" s="11"/>
     </row>
-    <row r="121" spans="1:22" ht="27" thickBot="1">
+    <row r="121" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A121" s="12"/>
       <c r="B121" s="6">
         <v>46050.546689814815</v>
@@ -9219,7 +9219,7 @@
       <c r="U121" s="11"/>
       <c r="V121" s="11"/>
     </row>
-    <row r="122" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="122" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A122" s="5"/>
       <c r="B122" s="6">
         <v>46050.606516203705</v>
@@ -9273,7 +9273,7 @@
       <c r="U122" s="11"/>
       <c r="V122" s="11"/>
     </row>
-    <row r="123" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="123" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A123" s="12"/>
       <c r="B123" s="6">
         <v>46050.763807870368</v>
@@ -9319,7 +9319,7 @@
       <c r="U123" s="11"/>
       <c r="V123" s="11"/>
     </row>
-    <row r="124" spans="1:22" ht="27" thickBot="1">
+    <row r="124" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A124" s="5"/>
       <c r="B124" s="6">
         <v>46051.481249999997</v>
@@ -9365,7 +9365,7 @@
       <c r="U124" s="11"/>
       <c r="V124" s="11"/>
     </row>
-    <row r="125" spans="1:22" ht="27" thickBot="1">
+    <row r="125" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A125" s="12"/>
       <c r="B125" s="6">
         <v>46051.651400462964</v>
@@ -9411,7 +9411,7 @@
       <c r="U125" s="11"/>
       <c r="V125" s="11"/>
     </row>
-    <row r="126" spans="1:22" ht="27" thickBot="1">
+    <row r="126" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A126" s="5"/>
       <c r="B126" s="6">
         <v>46056.336643518516</v>
@@ -9457,7 +9457,7 @@
       <c r="U126" s="11"/>
       <c r="V126" s="11"/>
     </row>
-    <row r="127" spans="1:22" ht="27" thickBot="1">
+    <row r="127" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A127" s="12"/>
       <c r="B127" s="6">
         <v>46058.329814814817</v>
@@ -9511,7 +9511,7 @@
       <c r="U127" s="11"/>
       <c r="V127" s="11"/>
     </row>
-    <row r="128" spans="1:22" ht="27" thickBot="1">
+    <row r="128" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A128" s="5"/>
       <c r="B128" s="6">
         <v>46058.331157407411</v>
@@ -9565,7 +9565,7 @@
       <c r="U128" s="11"/>
       <c r="V128" s="11"/>
     </row>
-    <row r="129" spans="1:22" ht="27" thickBot="1">
+    <row r="129" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A129" s="12"/>
       <c r="B129" s="6">
         <v>46058.333460648151</v>
@@ -9611,7 +9611,7 @@
       <c r="U129" s="11"/>
       <c r="V129" s="11"/>
     </row>
-    <row r="130" spans="1:22" ht="27" thickBot="1">
+    <row r="130" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A130" s="5"/>
       <c r="B130" s="6">
         <v>46058.342129629629</v>
@@ -9657,7 +9657,7 @@
       <c r="U130" s="11"/>
       <c r="V130" s="11"/>
     </row>
-    <row r="131" spans="1:22" ht="27" thickBot="1">
+    <row r="131" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A131" s="12"/>
       <c r="B131" s="6">
         <v>46058.364699074074</v>
@@ -9703,7 +9703,7 @@
       <c r="U131" s="11"/>
       <c r="V131" s="11"/>
     </row>
-    <row r="132" spans="1:22" ht="27" thickBot="1">
+    <row r="132" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A132" s="5"/>
       <c r="B132" s="6">
         <v>46058.38853009259</v>
@@ -9757,7 +9757,7 @@
       <c r="U132" s="11"/>
       <c r="V132" s="11"/>
     </row>
-    <row r="133" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="133" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A133" s="12"/>
       <c r="B133" s="6">
         <v>46058.393854166665</v>
@@ -9811,7 +9811,7 @@
       <c r="U133" s="11"/>
       <c r="V133" s="11"/>
     </row>
-    <row r="134" spans="1:22" ht="27" thickBot="1">
+    <row r="134" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A134" s="5"/>
       <c r="B134" s="6">
         <v>46058.403356481482</v>
@@ -9865,7 +9865,7 @@
       <c r="U134" s="11"/>
       <c r="V134" s="11"/>
     </row>
-    <row r="135" spans="1:22" ht="27" thickBot="1">
+    <row r="135" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A135" s="12"/>
       <c r="B135" s="6">
         <v>46058.440949074073</v>
@@ -9911,7 +9911,7 @@
       <c r="U135" s="11"/>
       <c r="V135" s="11"/>
     </row>
-    <row r="136" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="136" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A136" s="5"/>
       <c r="B136" s="6">
         <v>46058.443368055552</v>
@@ -9965,7 +9965,7 @@
       <c r="U136" s="11"/>
       <c r="V136" s="11"/>
     </row>
-    <row r="137" spans="1:22" ht="27" thickBot="1">
+    <row r="137" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A137" s="12"/>
       <c r="B137" s="6">
         <v>46058.454375000001</v>
@@ -10011,7 +10011,7 @@
       <c r="U137" s="11"/>
       <c r="V137" s="11"/>
     </row>
-    <row r="138" spans="1:22" ht="27" thickBot="1">
+    <row r="138" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A138" s="5"/>
       <c r="B138" s="6">
         <v>46058.457152777781</v>
@@ -10057,7 +10057,7 @@
       <c r="U138" s="11"/>
       <c r="V138" s="11"/>
     </row>
-    <row r="139" spans="1:22" ht="27" thickBot="1">
+    <row r="139" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A139" s="12"/>
       <c r="B139" s="6">
         <v>46058.589421296296</v>
@@ -10103,7 +10103,7 @@
       <c r="U139" s="11"/>
       <c r="V139" s="11"/>
     </row>
-    <row r="140" spans="1:22" ht="27" thickBot="1">
+    <row r="140" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A140" s="5"/>
       <c r="B140" s="6">
         <v>46058.591319444444</v>
@@ -10157,7 +10157,7 @@
       <c r="U140" s="11"/>
       <c r="V140" s="11"/>
     </row>
-    <row r="141" spans="1:22" ht="53.4" thickBot="1">
+    <row r="141" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A141" s="12"/>
       <c r="B141" s="6">
         <v>46058.702152777776</v>
@@ -10211,7 +10211,7 @@
       <c r="U141" s="11"/>
       <c r="V141" s="11"/>
     </row>
-    <row r="142" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="142" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A142" s="5"/>
       <c r="B142" s="6">
         <v>46058.737847222219</v>
@@ -10265,7 +10265,7 @@
       <c r="U142" s="11"/>
       <c r="V142" s="11"/>
     </row>
-    <row r="143" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="143" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A143" s="12"/>
       <c r="B143" s="6">
         <v>46058.802395833336</v>
@@ -10319,7 +10319,7 @@
       <c r="U143" s="11"/>
       <c r="V143" s="11"/>
     </row>
-    <row r="144" spans="1:22" ht="27" thickBot="1">
+    <row r="144" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A144" s="5"/>
       <c r="B144" s="6">
         <v>46058.836041666669</v>
@@ -10373,7 +10373,7 @@
       <c r="U144" s="11"/>
       <c r="V144" s="11"/>
     </row>
-    <row r="145" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="145" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A145" s="34"/>
       <c r="B145" s="35">
         <v>46058.863032407404</v>
@@ -10427,7 +10427,7 @@
       <c r="U145" s="11"/>
       <c r="V145" s="11"/>
     </row>
-    <row r="146" spans="1:22" ht="27" thickBot="1">
+    <row r="146" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A146" s="5"/>
       <c r="B146" s="6">
         <v>46058.898275462961</v>
@@ -10481,7 +10481,7 @@
       <c r="U146" s="11"/>
       <c r="V146" s="11"/>
     </row>
-    <row r="147" spans="1:22" ht="27" thickBot="1">
+    <row r="147" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A147" s="12"/>
       <c r="B147" s="6">
         <v>46058.914259259262</v>
@@ -10527,7 +10527,7 @@
       <c r="U147" s="11"/>
       <c r="V147" s="11"/>
     </row>
-    <row r="148" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="148" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A148" s="5"/>
       <c r="B148" s="6">
         <v>46058.94021990741</v>
@@ -10581,7 +10581,7 @@
       <c r="U148" s="11"/>
       <c r="V148" s="11"/>
     </row>
-    <row r="149" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="149" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A149" s="12"/>
       <c r="B149" s="6">
         <v>46059.478587962964</v>
@@ -10635,7 +10635,7 @@
       <c r="U149" s="11"/>
       <c r="V149" s="11"/>
     </row>
-    <row r="150" spans="1:22" ht="27" thickBot="1">
+    <row r="150" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A150" s="5"/>
       <c r="B150" s="6">
         <v>46059.633344907408</v>
@@ -10681,7 +10681,7 @@
       <c r="U150" s="11"/>
       <c r="V150" s="11"/>
     </row>
-    <row r="151" spans="1:22" ht="53.4" thickBot="1">
+    <row r="151" spans="1:22" ht="52.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A151" s="12"/>
       <c r="B151" s="6">
         <v>46059.675925925927</v>
@@ -10735,7 +10735,7 @@
       <c r="U151" s="11"/>
       <c r="V151" s="11"/>
     </row>
-    <row r="152" spans="1:22" ht="40.200000000000003" thickBot="1">
+    <row r="152" spans="1:22" ht="39.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A152" s="5"/>
       <c r="B152" s="6">
         <v>46062.374236111114</v>
@@ -10789,7 +10789,7 @@
       <c r="U152" s="11"/>
       <c r="V152" s="11"/>
     </row>
-    <row r="153" spans="1:22" ht="27" thickBot="1">
+    <row r="153" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A153" s="34"/>
       <c r="B153" s="35">
         <v>46062.418194444443</v>
@@ -10835,7 +10835,7 @@
       <c r="U153" s="11"/>
       <c r="V153" s="11"/>
     </row>
-    <row r="154" spans="1:22" ht="27" thickBot="1">
+    <row r="154" spans="1:22" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A154" s="49"/>
       <c r="B154" s="50">
         <v>46062.669456018521</v>
@@ -10881,7 +10881,7 @@
       <c r="U154" s="11"/>
       <c r="V154" s="11"/>
     </row>
-    <row r="155" spans="1:22" ht="14.4" thickBot="1">
+    <row r="155" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A155" s="11"/>
       <c r="B155" s="11"/>
       <c r="C155" s="11"/>
@@ -10905,7 +10905,7 @@
       <c r="U155" s="11"/>
       <c r="V155" s="11"/>
     </row>
-    <row r="156" spans="1:22" ht="14.4" thickBot="1">
+    <row r="156" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A156" s="11"/>
       <c r="B156" s="11"/>
       <c r="C156" s="11"/>
@@ -10929,7 +10929,7 @@
       <c r="U156" s="11"/>
       <c r="V156" s="11"/>
     </row>
-    <row r="157" spans="1:22" ht="14.4" thickBot="1">
+    <row r="157" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A157" s="11"/>
       <c r="B157" s="11"/>
       <c r="C157" s="11"/>
@@ -10953,7 +10953,7 @@
       <c r="U157" s="11"/>
       <c r="V157" s="11"/>
     </row>
-    <row r="158" spans="1:22" ht="14.4" thickBot="1">
+    <row r="158" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A158" s="11"/>
       <c r="B158" s="11"/>
       <c r="C158" s="11"/>
@@ -10977,7 +10977,7 @@
       <c r="U158" s="11"/>
       <c r="V158" s="11"/>
     </row>
-    <row r="159" spans="1:22" ht="14.4" thickBot="1">
+    <row r="159" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A159" s="11"/>
       <c r="B159" s="11"/>
       <c r="C159" s="11"/>
@@ -11001,7 +11001,7 @@
       <c r="U159" s="11"/>
       <c r="V159" s="11"/>
     </row>
-    <row r="160" spans="1:22" ht="14.4" thickBot="1">
+    <row r="160" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A160" s="11"/>
       <c r="B160" s="11"/>
       <c r="C160" s="11"/>
@@ -11025,7 +11025,7 @@
       <c r="U160" s="11"/>
       <c r="V160" s="11"/>
     </row>
-    <row r="161" spans="1:22" ht="14.4" thickBot="1">
+    <row r="161" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A161" s="11"/>
       <c r="B161" s="11"/>
       <c r="C161" s="11"/>
@@ -11049,7 +11049,7 @@
       <c r="U161" s="11"/>
       <c r="V161" s="11"/>
     </row>
-    <row r="162" spans="1:22" ht="14.4" thickBot="1">
+    <row r="162" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A162" s="11"/>
       <c r="B162" s="11"/>
       <c r="C162" s="11"/>
@@ -11073,7 +11073,7 @@
       <c r="U162" s="11"/>
       <c r="V162" s="11"/>
     </row>
-    <row r="163" spans="1:22" ht="14.4" thickBot="1">
+    <row r="163" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A163" s="11"/>
       <c r="B163" s="11"/>
       <c r="C163" s="11"/>
@@ -11097,7 +11097,7 @@
       <c r="U163" s="11"/>
       <c r="V163" s="11"/>
     </row>
-    <row r="164" spans="1:22" ht="14.4" thickBot="1">
+    <row r="164" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A164" s="11"/>
       <c r="B164" s="11"/>
       <c r="C164" s="11"/>
@@ -11121,7 +11121,7 @@
       <c r="U164" s="11"/>
       <c r="V164" s="11"/>
     </row>
-    <row r="165" spans="1:22" ht="14.4" thickBot="1">
+    <row r="165" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A165" s="11"/>
       <c r="B165" s="11"/>
       <c r="C165" s="11"/>
@@ -11145,7 +11145,7 @@
       <c r="U165" s="11"/>
       <c r="V165" s="11"/>
     </row>
-    <row r="166" spans="1:22" ht="14.4" thickBot="1">
+    <row r="166" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A166" s="11"/>
       <c r="B166" s="11"/>
       <c r="C166" s="11"/>
@@ -11169,7 +11169,7 @@
       <c r="U166" s="11"/>
       <c r="V166" s="11"/>
     </row>
-    <row r="167" spans="1:22" ht="14.4" thickBot="1">
+    <row r="167" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A167" s="11"/>
       <c r="B167" s="11"/>
       <c r="C167" s="11"/>
@@ -11193,7 +11193,7 @@
       <c r="U167" s="11"/>
       <c r="V167" s="11"/>
     </row>
-    <row r="168" spans="1:22" ht="14.4" thickBot="1">
+    <row r="168" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A168" s="11"/>
       <c r="B168" s="11"/>
       <c r="C168" s="11"/>
@@ -11217,7 +11217,7 @@
       <c r="U168" s="11"/>
       <c r="V168" s="11"/>
     </row>
-    <row r="169" spans="1:22" ht="14.4" thickBot="1">
+    <row r="169" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A169" s="11"/>
       <c r="B169" s="11"/>
       <c r="C169" s="11"/>
@@ -11241,7 +11241,7 @@
       <c r="U169" s="11"/>
       <c r="V169" s="11"/>
     </row>
-    <row r="170" spans="1:22" ht="14.4" thickBot="1">
+    <row r="170" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A170" s="11"/>
       <c r="B170" s="11"/>
       <c r="C170" s="11"/>
@@ -11265,7 +11265,7 @@
       <c r="U170" s="11"/>
       <c r="V170" s="11"/>
     </row>
-    <row r="171" spans="1:22" ht="14.4" thickBot="1">
+    <row r="171" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A171" s="11"/>
       <c r="B171" s="11"/>
       <c r="C171" s="11"/>
@@ -11289,7 +11289,7 @@
       <c r="U171" s="11"/>
       <c r="V171" s="11"/>
     </row>
-    <row r="172" spans="1:22" ht="14.4" thickBot="1">
+    <row r="172" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A172" s="11"/>
       <c r="B172" s="11"/>
       <c r="C172" s="11"/>
@@ -11313,7 +11313,7 @@
       <c r="U172" s="11"/>
       <c r="V172" s="11"/>
     </row>
-    <row r="173" spans="1:22" ht="14.4" thickBot="1">
+    <row r="173" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A173" s="11"/>
       <c r="B173" s="11"/>
       <c r="C173" s="11"/>
@@ -11337,7 +11337,7 @@
       <c r="U173" s="11"/>
       <c r="V173" s="11"/>
     </row>
-    <row r="174" spans="1:22" ht="14.4" thickBot="1">
+    <row r="174" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A174" s="11"/>
       <c r="B174" s="11"/>
       <c r="C174" s="11"/>
@@ -11361,7 +11361,7 @@
       <c r="U174" s="11"/>
       <c r="V174" s="11"/>
     </row>
-    <row r="175" spans="1:22" ht="14.4" thickBot="1">
+    <row r="175" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A175" s="11"/>
       <c r="B175" s="11"/>
       <c r="C175" s="11"/>
@@ -11385,7 +11385,7 @@
       <c r="U175" s="11"/>
       <c r="V175" s="11"/>
     </row>
-    <row r="176" spans="1:22" ht="14.4" thickBot="1">
+    <row r="176" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A176" s="11"/>
       <c r="B176" s="11"/>
       <c r="C176" s="11"/>
@@ -11409,7 +11409,7 @@
       <c r="U176" s="11"/>
       <c r="V176" s="11"/>
     </row>
-    <row r="177" spans="1:22" ht="14.4" thickBot="1">
+    <row r="177" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A177" s="11"/>
       <c r="B177" s="11"/>
       <c r="C177" s="11"/>
@@ -11433,7 +11433,7 @@
       <c r="U177" s="11"/>
       <c r="V177" s="11"/>
     </row>
-    <row r="178" spans="1:22" ht="14.4" thickBot="1">
+    <row r="178" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A178" s="11"/>
       <c r="B178" s="11"/>
       <c r="C178" s="11"/>
@@ -11457,7 +11457,7 @@
       <c r="U178" s="11"/>
       <c r="V178" s="11"/>
     </row>
-    <row r="179" spans="1:22" ht="14.4" thickBot="1">
+    <row r="179" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A179" s="11"/>
       <c r="B179" s="11"/>
       <c r="C179" s="11"/>
@@ -11481,7 +11481,7 @@
       <c r="U179" s="11"/>
       <c r="V179" s="11"/>
     </row>
-    <row r="180" spans="1:22" ht="14.4" thickBot="1">
+    <row r="180" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A180" s="11"/>
       <c r="B180" s="11"/>
       <c r="C180" s="11"/>
@@ -11505,7 +11505,7 @@
       <c r="U180" s="11"/>
       <c r="V180" s="11"/>
     </row>
-    <row r="181" spans="1:22" ht="14.4" thickBot="1">
+    <row r="181" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A181" s="11"/>
       <c r="B181" s="11"/>
       <c r="C181" s="11"/>
@@ -11529,7 +11529,7 @@
       <c r="U181" s="11"/>
       <c r="V181" s="11"/>
     </row>
-    <row r="182" spans="1:22" ht="14.4" thickBot="1">
+    <row r="182" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A182" s="11"/>
       <c r="B182" s="11"/>
       <c r="C182" s="11"/>
@@ -11553,7 +11553,7 @@
       <c r="U182" s="11"/>
       <c r="V182" s="11"/>
     </row>
-    <row r="183" spans="1:22" ht="14.4" thickBot="1">
+    <row r="183" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A183" s="11"/>
       <c r="B183" s="11"/>
       <c r="C183" s="11"/>
@@ -11577,7 +11577,7 @@
       <c r="U183" s="11"/>
       <c r="V183" s="11"/>
     </row>
-    <row r="184" spans="1:22" ht="14.4" thickBot="1">
+    <row r="184" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A184" s="11"/>
       <c r="B184" s="11"/>
       <c r="C184" s="11"/>
@@ -11601,7 +11601,7 @@
       <c r="U184" s="11"/>
       <c r="V184" s="11"/>
     </row>
-    <row r="185" spans="1:22" ht="14.4" thickBot="1">
+    <row r="185" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A185" s="11"/>
       <c r="B185" s="11"/>
       <c r="C185" s="11"/>
@@ -11625,7 +11625,7 @@
       <c r="U185" s="11"/>
       <c r="V185" s="11"/>
     </row>
-    <row r="186" spans="1:22" ht="14.4" thickBot="1">
+    <row r="186" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A186" s="11"/>
       <c r="B186" s="11"/>
       <c r="C186" s="11"/>
@@ -11649,7 +11649,7 @@
       <c r="U186" s="11"/>
       <c r="V186" s="11"/>
     </row>
-    <row r="187" spans="1:22" ht="14.4" thickBot="1">
+    <row r="187" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A187" s="11"/>
       <c r="B187" s="11"/>
       <c r="C187" s="11"/>
@@ -11673,7 +11673,7 @@
       <c r="U187" s="11"/>
       <c r="V187" s="11"/>
     </row>
-    <row r="188" spans="1:22" ht="14.4" thickBot="1">
+    <row r="188" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A188" s="11"/>
       <c r="B188" s="11"/>
       <c r="C188" s="11"/>
@@ -11697,7 +11697,7 @@
       <c r="U188" s="11"/>
       <c r="V188" s="11"/>
     </row>
-    <row r="189" spans="1:22" ht="14.4" thickBot="1">
+    <row r="189" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A189" s="11"/>
       <c r="B189" s="11"/>
       <c r="C189" s="11"/>
@@ -11721,7 +11721,7 @@
       <c r="U189" s="11"/>
       <c r="V189" s="11"/>
     </row>
-    <row r="190" spans="1:22" ht="14.4" thickBot="1">
+    <row r="190" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A190" s="11"/>
       <c r="B190" s="11"/>
       <c r="C190" s="11"/>
@@ -11745,7 +11745,7 @@
       <c r="U190" s="11"/>
       <c r="V190" s="11"/>
     </row>
-    <row r="191" spans="1:22" ht="14.4" thickBot="1">
+    <row r="191" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A191" s="11"/>
       <c r="B191" s="11"/>
       <c r="C191" s="11"/>
@@ -11769,7 +11769,7 @@
       <c r="U191" s="11"/>
       <c r="V191" s="11"/>
     </row>
-    <row r="192" spans="1:22" ht="14.4" thickBot="1">
+    <row r="192" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A192" s="11"/>
       <c r="B192" s="11"/>
       <c r="C192" s="11"/>
@@ -11793,7 +11793,7 @@
       <c r="U192" s="11"/>
       <c r="V192" s="11"/>
     </row>
-    <row r="193" spans="1:22" ht="14.4" thickBot="1">
+    <row r="193" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A193" s="11"/>
       <c r="B193" s="11"/>
       <c r="C193" s="11"/>
@@ -11817,7 +11817,7 @@
       <c r="U193" s="11"/>
       <c r="V193" s="11"/>
     </row>
-    <row r="194" spans="1:22" ht="14.4" thickBot="1">
+    <row r="194" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A194" s="11"/>
       <c r="B194" s="11"/>
       <c r="C194" s="11"/>
@@ -11841,7 +11841,7 @@
       <c r="U194" s="11"/>
       <c r="V194" s="11"/>
     </row>
-    <row r="195" spans="1:22" ht="14.4" thickBot="1">
+    <row r="195" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A195" s="11"/>
       <c r="B195" s="11"/>
       <c r="C195" s="11"/>
@@ -11865,7 +11865,7 @@
       <c r="U195" s="11"/>
       <c r="V195" s="11"/>
     </row>
-    <row r="196" spans="1:22" ht="14.4" thickBot="1">
+    <row r="196" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A196" s="11"/>
       <c r="B196" s="11"/>
       <c r="C196" s="11"/>
@@ -11889,7 +11889,7 @@
       <c r="U196" s="11"/>
       <c r="V196" s="11"/>
     </row>
-    <row r="197" spans="1:22" ht="14.4" thickBot="1">
+    <row r="197" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A197" s="11"/>
       <c r="B197" s="11"/>
       <c r="C197" s="11"/>
@@ -11913,7 +11913,7 @@
       <c r="U197" s="11"/>
       <c r="V197" s="11"/>
     </row>
-    <row r="198" spans="1:22" ht="14.4" thickBot="1">
+    <row r="198" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A198" s="11"/>
       <c r="B198" s="11"/>
       <c r="C198" s="11"/>
@@ -11937,7 +11937,7 @@
       <c r="U198" s="11"/>
       <c r="V198" s="11"/>
     </row>
-    <row r="199" spans="1:22" ht="14.4" thickBot="1">
+    <row r="199" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A199" s="11"/>
       <c r="B199" s="11"/>
       <c r="C199" s="11"/>
@@ -11961,7 +11961,7 @@
       <c r="U199" s="11"/>
       <c r="V199" s="11"/>
     </row>
-    <row r="200" spans="1:22" ht="14.4" thickBot="1">
+    <row r="200" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A200" s="11"/>
       <c r="B200" s="11"/>
       <c r="C200" s="11"/>
@@ -11985,7 +11985,7 @@
       <c r="U200" s="11"/>
       <c r="V200" s="11"/>
     </row>
-    <row r="201" spans="1:22" ht="14.4" thickBot="1">
+    <row r="201" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A201" s="11"/>
       <c r="B201" s="11"/>
       <c r="C201" s="11"/>
@@ -12009,7 +12009,7 @@
       <c r="U201" s="11"/>
       <c r="V201" s="11"/>
     </row>
-    <row r="202" spans="1:22" ht="14.4" thickBot="1">
+    <row r="202" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A202" s="11"/>
       <c r="B202" s="11"/>
       <c r="C202" s="11"/>
@@ -12033,7 +12033,7 @@
       <c r="U202" s="11"/>
       <c r="V202" s="11"/>
     </row>
-    <row r="203" spans="1:22" ht="14.4" thickBot="1">
+    <row r="203" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A203" s="11"/>
       <c r="B203" s="11"/>
       <c r="C203" s="11"/>
@@ -12057,7 +12057,7 @@
       <c r="U203" s="11"/>
       <c r="V203" s="11"/>
     </row>
-    <row r="204" spans="1:22" ht="14.4" thickBot="1">
+    <row r="204" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A204" s="11"/>
       <c r="B204" s="11"/>
       <c r="C204" s="11"/>
@@ -12081,7 +12081,7 @@
       <c r="U204" s="11"/>
       <c r="V204" s="11"/>
     </row>
-    <row r="205" spans="1:22" ht="14.4" thickBot="1">
+    <row r="205" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A205" s="11"/>
       <c r="B205" s="11"/>
       <c r="C205" s="11"/>
@@ -12105,7 +12105,7 @@
       <c r="U205" s="11"/>
       <c r="V205" s="11"/>
     </row>
-    <row r="206" spans="1:22" ht="14.4" thickBot="1">
+    <row r="206" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A206" s="11"/>
       <c r="B206" s="11"/>
       <c r="C206" s="11"/>
@@ -12129,7 +12129,7 @@
       <c r="U206" s="11"/>
       <c r="V206" s="11"/>
     </row>
-    <row r="207" spans="1:22" ht="14.4" thickBot="1">
+    <row r="207" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A207" s="11"/>
       <c r="B207" s="11"/>
       <c r="C207" s="11"/>
@@ -12153,7 +12153,7 @@
       <c r="U207" s="11"/>
       <c r="V207" s="11"/>
     </row>
-    <row r="208" spans="1:22" ht="14.4" thickBot="1">
+    <row r="208" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A208" s="11"/>
       <c r="B208" s="11"/>
       <c r="C208" s="11"/>
@@ -12177,7 +12177,7 @@
       <c r="U208" s="11"/>
       <c r="V208" s="11"/>
     </row>
-    <row r="209" spans="1:22" ht="14.4" thickBot="1">
+    <row r="209" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A209" s="11"/>
       <c r="B209" s="11"/>
       <c r="C209" s="11"/>
@@ -12201,7 +12201,7 @@
       <c r="U209" s="11"/>
       <c r="V209" s="11"/>
     </row>
-    <row r="210" spans="1:22" ht="14.4" thickBot="1">
+    <row r="210" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A210" s="11"/>
       <c r="B210" s="11"/>
       <c r="C210" s="11"/>
@@ -12225,7 +12225,7 @@
       <c r="U210" s="11"/>
       <c r="V210" s="11"/>
     </row>
-    <row r="211" spans="1:22" ht="14.4" thickBot="1">
+    <row r="211" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A211" s="11"/>
       <c r="B211" s="11"/>
       <c r="C211" s="11"/>
@@ -12249,7 +12249,7 @@
       <c r="U211" s="11"/>
       <c r="V211" s="11"/>
     </row>
-    <row r="212" spans="1:22" ht="14.4" thickBot="1">
+    <row r="212" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A212" s="11"/>
       <c r="B212" s="11"/>
       <c r="C212" s="11"/>
@@ -12273,7 +12273,7 @@
       <c r="U212" s="11"/>
       <c r="V212" s="11"/>
     </row>
-    <row r="213" spans="1:22" ht="14.4" thickBot="1">
+    <row r="213" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A213" s="11"/>
       <c r="B213" s="11"/>
       <c r="C213" s="11"/>
@@ -12297,7 +12297,7 @@
       <c r="U213" s="11"/>
       <c r="V213" s="11"/>
     </row>
-    <row r="214" spans="1:22" ht="14.4" thickBot="1">
+    <row r="214" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A214" s="11"/>
       <c r="B214" s="11"/>
       <c r="C214" s="11"/>
@@ -12321,7 +12321,7 @@
       <c r="U214" s="11"/>
       <c r="V214" s="11"/>
     </row>
-    <row r="215" spans="1:22" ht="14.4" thickBot="1">
+    <row r="215" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A215" s="11"/>
       <c r="B215" s="11"/>
       <c r="C215" s="11"/>
@@ -12345,7 +12345,7 @@
       <c r="U215" s="11"/>
       <c r="V215" s="11"/>
     </row>
-    <row r="216" spans="1:22" ht="14.4" thickBot="1">
+    <row r="216" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A216" s="11"/>
       <c r="B216" s="11"/>
       <c r="C216" s="11"/>
@@ -12369,7 +12369,7 @@
       <c r="U216" s="11"/>
       <c r="V216" s="11"/>
     </row>
-    <row r="217" spans="1:22" ht="14.4" thickBot="1">
+    <row r="217" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A217" s="11"/>
       <c r="B217" s="11"/>
       <c r="C217" s="11"/>
@@ -12393,7 +12393,7 @@
       <c r="U217" s="11"/>
       <c r="V217" s="11"/>
     </row>
-    <row r="218" spans="1:22" ht="14.4" thickBot="1">
+    <row r="218" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A218" s="11"/>
       <c r="B218" s="11"/>
       <c r="C218" s="11"/>
@@ -12417,7 +12417,7 @@
       <c r="U218" s="11"/>
       <c r="V218" s="11"/>
     </row>
-    <row r="219" spans="1:22" ht="14.4" thickBot="1">
+    <row r="219" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A219" s="11"/>
       <c r="B219" s="11"/>
       <c r="C219" s="11"/>
@@ -12441,7 +12441,7 @@
       <c r="U219" s="11"/>
       <c r="V219" s="11"/>
     </row>
-    <row r="220" spans="1:22" ht="14.4" thickBot="1">
+    <row r="220" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A220" s="11"/>
       <c r="B220" s="11"/>
       <c r="C220" s="11"/>
@@ -12465,7 +12465,7 @@
       <c r="U220" s="11"/>
       <c r="V220" s="11"/>
     </row>
-    <row r="221" spans="1:22" ht="14.4" thickBot="1">
+    <row r="221" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A221" s="11"/>
       <c r="B221" s="11"/>
       <c r="C221" s="11"/>
@@ -12489,7 +12489,7 @@
       <c r="U221" s="11"/>
       <c r="V221" s="11"/>
     </row>
-    <row r="222" spans="1:22" ht="14.4" thickBot="1">
+    <row r="222" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A222" s="11"/>
       <c r="B222" s="11"/>
       <c r="C222" s="11"/>
@@ -12513,7 +12513,7 @@
       <c r="U222" s="11"/>
       <c r="V222" s="11"/>
     </row>
-    <row r="223" spans="1:22" ht="14.4" thickBot="1">
+    <row r="223" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A223" s="11"/>
       <c r="B223" s="11"/>
       <c r="C223" s="11"/>
@@ -12537,7 +12537,7 @@
       <c r="U223" s="11"/>
       <c r="V223" s="11"/>
     </row>
-    <row r="224" spans="1:22" ht="14.4" thickBot="1">
+    <row r="224" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A224" s="11"/>
       <c r="B224" s="11"/>
       <c r="C224" s="11"/>
@@ -12561,7 +12561,7 @@
       <c r="U224" s="11"/>
       <c r="V224" s="11"/>
     </row>
-    <row r="225" spans="1:22" ht="14.4" thickBot="1">
+    <row r="225" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A225" s="11"/>
       <c r="B225" s="11"/>
       <c r="C225" s="11"/>
@@ -12585,7 +12585,7 @@
       <c r="U225" s="11"/>
       <c r="V225" s="11"/>
     </row>
-    <row r="226" spans="1:22" ht="14.4" thickBot="1">
+    <row r="226" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A226" s="11"/>
       <c r="B226" s="11"/>
       <c r="C226" s="11"/>
@@ -12609,7 +12609,7 @@
       <c r="U226" s="11"/>
       <c r="V226" s="11"/>
     </row>
-    <row r="227" spans="1:22" ht="14.4" thickBot="1">
+    <row r="227" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A227" s="11"/>
       <c r="B227" s="11"/>
       <c r="C227" s="11"/>
@@ -12633,7 +12633,7 @@
       <c r="U227" s="11"/>
       <c r="V227" s="11"/>
     </row>
-    <row r="228" spans="1:22" ht="14.4" thickBot="1">
+    <row r="228" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A228" s="11"/>
       <c r="B228" s="11"/>
       <c r="C228" s="11"/>
@@ -12657,7 +12657,7 @@
       <c r="U228" s="11"/>
       <c r="V228" s="11"/>
     </row>
-    <row r="229" spans="1:22" ht="14.4" thickBot="1">
+    <row r="229" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A229" s="11"/>
       <c r="B229" s="11"/>
       <c r="C229" s="11"/>
@@ -12681,7 +12681,7 @@
       <c r="U229" s="11"/>
       <c r="V229" s="11"/>
     </row>
-    <row r="230" spans="1:22" ht="14.4" thickBot="1">
+    <row r="230" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A230" s="11"/>
       <c r="B230" s="11"/>
       <c r="C230" s="11"/>
@@ -12705,7 +12705,7 @@
       <c r="U230" s="11"/>
       <c r="V230" s="11"/>
     </row>
-    <row r="231" spans="1:22" ht="14.4" thickBot="1">
+    <row r="231" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A231" s="11"/>
       <c r="B231" s="11"/>
       <c r="C231" s="11"/>
@@ -12729,7 +12729,7 @@
       <c r="U231" s="11"/>
       <c r="V231" s="11"/>
     </row>
-    <row r="232" spans="1:22" ht="14.4" thickBot="1">
+    <row r="232" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A232" s="11"/>
       <c r="B232" s="11"/>
       <c r="C232" s="11"/>
@@ -12753,7 +12753,7 @@
       <c r="U232" s="11"/>
       <c r="V232" s="11"/>
     </row>
-    <row r="233" spans="1:22" ht="14.4" thickBot="1">
+    <row r="233" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A233" s="11"/>
       <c r="B233" s="11"/>
       <c r="C233" s="11"/>
@@ -12777,7 +12777,7 @@
       <c r="U233" s="11"/>
       <c r="V233" s="11"/>
     </row>
-    <row r="234" spans="1:22" ht="14.4" thickBot="1">
+    <row r="234" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A234" s="11"/>
       <c r="B234" s="11"/>
       <c r="C234" s="11"/>
@@ -12801,7 +12801,7 @@
       <c r="U234" s="11"/>
       <c r="V234" s="11"/>
     </row>
-    <row r="235" spans="1:22" ht="14.4" thickBot="1">
+    <row r="235" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A235" s="11"/>
       <c r="B235" s="11"/>
       <c r="C235" s="11"/>
@@ -12825,7 +12825,7 @@
       <c r="U235" s="11"/>
       <c r="V235" s="11"/>
     </row>
-    <row r="236" spans="1:22" ht="14.4" thickBot="1">
+    <row r="236" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A236" s="11"/>
       <c r="B236" s="11"/>
       <c r="C236" s="11"/>
@@ -12849,7 +12849,7 @@
       <c r="U236" s="11"/>
       <c r="V236" s="11"/>
     </row>
-    <row r="237" spans="1:22" ht="14.4" thickBot="1">
+    <row r="237" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A237" s="11"/>
       <c r="B237" s="11"/>
       <c r="C237" s="11"/>
@@ -12873,7 +12873,7 @@
       <c r="U237" s="11"/>
       <c r="V237" s="11"/>
     </row>
-    <row r="238" spans="1:22" ht="14.4" thickBot="1">
+    <row r="238" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A238" s="11"/>
       <c r="B238" s="11"/>
       <c r="C238" s="11"/>
@@ -12897,7 +12897,7 @@
       <c r="U238" s="11"/>
       <c r="V238" s="11"/>
     </row>
-    <row r="239" spans="1:22" ht="14.4" thickBot="1">
+    <row r="239" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A239" s="11"/>
       <c r="B239" s="11"/>
       <c r="C239" s="11"/>
@@ -12921,7 +12921,7 @@
       <c r="U239" s="11"/>
       <c r="V239" s="11"/>
     </row>
-    <row r="240" spans="1:22" ht="14.4" thickBot="1">
+    <row r="240" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A240" s="11"/>
       <c r="B240" s="11"/>
       <c r="C240" s="11"/>
@@ -12945,7 +12945,7 @@
       <c r="U240" s="11"/>
       <c r="V240" s="11"/>
     </row>
-    <row r="241" spans="1:22" ht="14.4" thickBot="1">
+    <row r="241" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A241" s="11"/>
       <c r="B241" s="11"/>
       <c r="C241" s="11"/>
@@ -12969,7 +12969,7 @@
       <c r="U241" s="11"/>
       <c r="V241" s="11"/>
     </row>
-    <row r="242" spans="1:22" ht="14.4" thickBot="1">
+    <row r="242" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A242" s="11"/>
       <c r="B242" s="11"/>
       <c r="C242" s="11"/>
@@ -12993,7 +12993,7 @@
       <c r="U242" s="11"/>
       <c r="V242" s="11"/>
     </row>
-    <row r="243" spans="1:22" ht="14.4" thickBot="1">
+    <row r="243" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A243" s="11"/>
       <c r="B243" s="11"/>
       <c r="C243" s="11"/>
@@ -13017,7 +13017,7 @@
       <c r="U243" s="11"/>
       <c r="V243" s="11"/>
     </row>
-    <row r="244" spans="1:22" ht="14.4" thickBot="1">
+    <row r="244" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A244" s="11"/>
       <c r="B244" s="11"/>
       <c r="C244" s="11"/>
@@ -13041,7 +13041,7 @@
       <c r="U244" s="11"/>
       <c r="V244" s="11"/>
     </row>
-    <row r="245" spans="1:22" ht="14.4" thickBot="1">
+    <row r="245" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A245" s="11"/>
       <c r="B245" s="11"/>
       <c r="C245" s="11"/>
@@ -13065,7 +13065,7 @@
       <c r="U245" s="11"/>
       <c r="V245" s="11"/>
     </row>
-    <row r="246" spans="1:22" ht="14.4" thickBot="1">
+    <row r="246" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A246" s="11"/>
       <c r="B246" s="11"/>
       <c r="C246" s="11"/>
@@ -13089,7 +13089,7 @@
       <c r="U246" s="11"/>
       <c r="V246" s="11"/>
     </row>
-    <row r="247" spans="1:22" ht="14.4" thickBot="1">
+    <row r="247" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A247" s="11"/>
       <c r="B247" s="11"/>
       <c r="C247" s="11"/>
@@ -13113,7 +13113,7 @@
       <c r="U247" s="11"/>
       <c r="V247" s="11"/>
     </row>
-    <row r="248" spans="1:22" ht="14.4" thickBot="1">
+    <row r="248" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A248" s="11"/>
       <c r="B248" s="11"/>
       <c r="C248" s="11"/>
@@ -13137,7 +13137,7 @@
       <c r="U248" s="11"/>
       <c r="V248" s="11"/>
     </row>
-    <row r="249" spans="1:22" ht="14.4" thickBot="1">
+    <row r="249" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A249" s="11"/>
       <c r="B249" s="11"/>
       <c r="C249" s="11"/>
@@ -13161,7 +13161,7 @@
       <c r="U249" s="11"/>
       <c r="V249" s="11"/>
     </row>
-    <row r="250" spans="1:22" ht="14.4" thickBot="1">
+    <row r="250" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A250" s="11"/>
       <c r="B250" s="11"/>
       <c r="C250" s="11"/>
@@ -13185,7 +13185,7 @@
       <c r="U250" s="11"/>
       <c r="V250" s="11"/>
     </row>
-    <row r="251" spans="1:22" ht="14.4" thickBot="1">
+    <row r="251" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A251" s="11"/>
       <c r="B251" s="11"/>
       <c r="C251" s="11"/>
@@ -13209,7 +13209,7 @@
       <c r="U251" s="11"/>
       <c r="V251" s="11"/>
     </row>
-    <row r="252" spans="1:22" ht="14.4" thickBot="1">
+    <row r="252" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A252" s="11"/>
       <c r="B252" s="11"/>
       <c r="C252" s="11"/>
@@ -13233,7 +13233,7 @@
       <c r="U252" s="11"/>
       <c r="V252" s="11"/>
     </row>
-    <row r="253" spans="1:22" ht="14.4" thickBot="1">
+    <row r="253" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A253" s="11"/>
       <c r="B253" s="11"/>
       <c r="C253" s="11"/>

</xml_diff>